<commit_message>
SCRUM-9 update passing test evidence after bug fixes
</commit_message>
<xml_diff>
--- a/docs/test_cases_patient_search.xlsx
+++ b/docs/test_cases_patient_search.xlsx
@@ -1203,12 +1203,12 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>ID 0 was accepted; no validation error appeared and 'No patients found.' was shown.</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>Patient ID 0 was rejected with 'Patient ID must be 1 or greater.'; no results were displayed.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>docs/screenshots/BUG_TC-S12_zero-id-accepted.png</t>
+          <t>docs/screenshots/FIXED_TC-S12_zero-id-rejected.png</t>
         </is>
       </c>
     </row>
@@ -1465,12 +1465,12 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>The 51-character name was accepted; no validation error appeared and 'No patients found.' was shown.</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>The 51-character name was rejected with 'Name must be between 2 and 50 characters.'; no results were displayed.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>docs/screenshots/BUG_TC-S18_name-51-accepted.png</t>
+          <t>docs/screenshots/FIXED_TC-S18_name-51-rejected.png</t>
         </is>
       </c>
     </row>
@@ -1512,12 +1512,12 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>No error appeared; all 6 seeded patient records were displayed.</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>'Enter a Patient ID or name.' was shown and no patient records were displayed.</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>docs/screenshots/BUG_TC-S19_empty-search-returns-all.png</t>
+          <t>docs/screenshots/FIXED_TC-S19_empty-search-rejected.png</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Whitespace was trimmed to empty, but no error appeared and all 6 records were displayed.</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>Whitespace was trimmed to empty; 'Enter a Patient ID or name.' was shown and no records were displayed.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>docs/screenshots/BUG_TC-S20_whitespace-search-returns-all.png</t>
+          <t>docs/screenshots/FIXED_TC-S20_whitespace-search-rejected.png</t>
         </is>
       </c>
     </row>
@@ -1649,12 +1649,12 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Only ravi singh was displayed; Ravi Kumar was omitted.</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>The lowercase search displayed both Ravi Kumar and ravi singh.</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>docs/screenshots/BUG_TC-S22_lowercase-search-case-sensitive.png</t>
+          <t>docs/screenshots/FIXED_TC-S22_lowercase-search.png</t>
         </is>
       </c>
     </row>
@@ -1696,12 +1696,12 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>No rows were displayed; 'No patients found.' was shown.</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>The uppercase search displayed both Ravi Kumar and ravi singh.</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>docs/screenshots/BUG_TC-S23_uppercase-search-case-sensitive.png</t>
+          <t>docs/screenshots/FIXED_TC-S23_uppercase-search.png</t>
         </is>
       </c>
     </row>
@@ -1743,12 +1743,12 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Only Ravi Kumar was displayed; ravi singh was omitted.</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>The title-case search displayed both Ravi Kumar and ravi singh.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>docs/screenshots/BUG_TC-S24_titlecase-search-case-sensitive.png</t>
+          <t>docs/screenshots/FIXED_TC-S24_titlecase-search.png</t>
         </is>
       </c>
     </row>

</xml_diff>